<commit_message>
user role landing page
</commit_message>
<xml_diff>
--- a/Documents/devfiles/excel/DevoloperActivities.xlsx
+++ b/Documents/devfiles/excel/DevoloperActivities.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitLab\joboffer\Documents\devfiles\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Gitlab\joboffer\Documents\devfiles\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79CA5BE6-ECE1-4EEC-AC32-76B91BF5A623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96BC441A-4112-48F2-8A9A-0DDB48FFF0B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{337275F3-F812-418C-B02B-6398BC7C9B39}"/>
+    <workbookView xWindow="-25260" yWindow="5445" windowWidth="23040" windowHeight="12120" activeTab="1" xr2:uid="{337275F3-F812-418C-B02B-6398BC7C9B39}"/>
   </bookViews>
   <sheets>
     <sheet name="Draft" sheetId="2" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="116">
   <si>
     <t>Daily sync of responses from MS forms to be scheduled at: 7AM, 12NN, 3PM</t>
   </si>
@@ -383,6 +383,24 @@
   </si>
   <si>
     <t>new password - hrodooffer@1</t>
+  </si>
+  <si>
+    <t>Manual Upload</t>
+  </si>
+  <si>
+    <t>Export</t>
+  </si>
+  <si>
+    <t>Remove Email Addres</t>
+  </si>
+  <si>
+    <t>Label "Dbox Sync"</t>
+  </si>
+  <si>
+    <t>Import Excel</t>
+  </si>
+  <si>
+    <t>Last Sync Date Time</t>
   </si>
 </sst>
 </file>
@@ -886,25 +904,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B9038A7-AD59-482A-8671-D3CB2D87EC41}">
   <dimension ref="B2:O8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="22.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.81640625" customWidth="1"/>
-    <col min="4" max="4" width="34.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.77734375" customWidth="1"/>
+    <col min="4" max="4" width="34.77734375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="32" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="46.08984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="30.1796875" customWidth="1"/>
-    <col min="8" max="8" width="37.7265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="27.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="46.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30.21875" customWidth="1"/>
+    <col min="8" max="8" width="37.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.6640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="25" customWidth="1"/>
     <col min="11" max="11" width="23" customWidth="1"/>
-    <col min="12" max="12" width="20.36328125" customWidth="1"/>
-    <col min="13" max="13" width="19.453125" customWidth="1"/>
-    <col min="14" max="14" width="28.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.33203125" customWidth="1"/>
+    <col min="13" max="13" width="19.44140625" customWidth="1"/>
+    <col min="14" max="14" width="28.77734375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
@@ -948,7 +966,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
@@ -992,7 +1010,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B4" s="2" t="s">
         <v>8</v>
       </c>
@@ -1021,7 +1039,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B5" s="2" t="s">
         <v>6</v>
       </c>
@@ -1041,7 +1059,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>9</v>
       </c>
@@ -1052,12 +1070,12 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B7" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B8" s="2" t="s">
         <v>49</v>
       </c>
@@ -1070,29 +1088,29 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EED69CB7-7627-4EC8-B1DF-810A0B37AA79}">
   <dimension ref="C1:Y26"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.36328125" customWidth="1"/>
-    <col min="2" max="2" width="11.26953125" customWidth="1"/>
-    <col min="3" max="3" width="62.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="63.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="46.7265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="63.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="28.90625" customWidth="1"/>
-    <col min="11" max="11" width="55.90625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="46.90625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="30.08984375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="90.1796875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="28.36328125" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="57.1796875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="19.6328125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="32.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.33203125" customWidth="1"/>
+    <col min="2" max="2" width="11.21875" customWidth="1"/>
+    <col min="3" max="3" width="66.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="63.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="46.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="63.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="28.88671875" customWidth="1"/>
+    <col min="11" max="11" width="55.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="46.88671875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="90.21875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="28.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="57.21875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="32.109375" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="33" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="31.6328125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="31.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:25" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="3:25" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C1" s="7">
         <v>46274</v>
       </c>
@@ -1163,7 +1181,7 @@
         <v>46296</v>
       </c>
     </row>
-    <row r="2" spans="3:25" x14ac:dyDescent="0.35">
+    <row r="2" spans="3:25" x14ac:dyDescent="0.3">
       <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1216,7 +1234,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="3:25" x14ac:dyDescent="0.35">
+    <row r="3" spans="3:25" x14ac:dyDescent="0.3">
       <c r="C3" t="s">
         <v>7</v>
       </c>
@@ -1251,7 +1269,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="3:25" x14ac:dyDescent="0.35">
+    <row r="4" spans="3:25" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
         <v>8</v>
       </c>
@@ -1286,7 +1304,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="3:25" x14ac:dyDescent="0.35">
+    <row r="5" spans="3:25" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
         <v>6</v>
       </c>
@@ -1324,7 +1342,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="6" spans="3:25" x14ac:dyDescent="0.35">
+    <row r="6" spans="3:25" x14ac:dyDescent="0.3">
       <c r="C6" t="s">
         <v>0</v>
       </c>
@@ -1344,10 +1362,13 @@
         <v>51</v>
       </c>
     </row>
-    <row r="7" spans="3:25" x14ac:dyDescent="0.35">
+    <row r="7" spans="3:25" x14ac:dyDescent="0.3">
       <c r="C7" t="s">
         <v>1</v>
       </c>
+      <c r="D7" t="s">
+        <v>110</v>
+      </c>
       <c r="E7" t="s">
         <v>61</v>
       </c>
@@ -1373,7 +1394,10 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="3:25" x14ac:dyDescent="0.35">
+    <row r="8" spans="3:25" x14ac:dyDescent="0.3">
+      <c r="D8" t="s">
+        <v>111</v>
+      </c>
       <c r="I8" t="s">
         <v>22</v>
       </c>
@@ -1390,7 +1414,10 @@
         <v>65</v>
       </c>
     </row>
-    <row r="9" spans="3:25" x14ac:dyDescent="0.35">
+    <row r="9" spans="3:25" x14ac:dyDescent="0.3">
+      <c r="D9" t="s">
+        <v>112</v>
+      </c>
       <c r="E9" t="s">
         <v>72</v>
       </c>
@@ -1406,8 +1433,14 @@
       <c r="O9" s="11" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="10" spans="3:25" x14ac:dyDescent="0.35">
+      <c r="Q9" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="10" spans="3:25" x14ac:dyDescent="0.3">
+      <c r="D10" t="s">
+        <v>113</v>
+      </c>
       <c r="E10" s="11" t="s">
         <v>73</v>
       </c>
@@ -1423,8 +1456,11 @@
       <c r="O10" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="11" spans="3:25" x14ac:dyDescent="0.35">
+      <c r="Q10" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="11" spans="3:25" x14ac:dyDescent="0.3">
       <c r="I11" t="s">
         <v>24</v>
       </c>
@@ -1434,8 +1470,11 @@
       <c r="O11" s="11" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="12" spans="3:25" x14ac:dyDescent="0.35">
+      <c r="Q11" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="12" spans="3:25" x14ac:dyDescent="0.3">
       <c r="E12" t="s">
         <v>74</v>
       </c>
@@ -1446,7 +1485,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="13" spans="3:25" x14ac:dyDescent="0.35">
+    <row r="13" spans="3:25" x14ac:dyDescent="0.3">
       <c r="E13" t="s">
         <v>75</v>
       </c>
@@ -1457,7 +1496,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="14" spans="3:25" x14ac:dyDescent="0.35">
+    <row r="14" spans="3:25" x14ac:dyDescent="0.3">
       <c r="E14" s="11" t="s">
         <v>76</v>
       </c>
@@ -1465,7 +1504,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="15" spans="3:25" x14ac:dyDescent="0.35">
+    <row r="15" spans="3:25" x14ac:dyDescent="0.3">
       <c r="E15" s="11" t="s">
         <v>77</v>
       </c>
@@ -1473,7 +1512,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="16" spans="3:25" x14ac:dyDescent="0.35">
+    <row r="16" spans="3:25" x14ac:dyDescent="0.3">
       <c r="E16" s="11" t="s">
         <v>78</v>
       </c>
@@ -1484,7 +1523,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="17" spans="5:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="5:9" x14ac:dyDescent="0.3">
       <c r="E17" s="11" t="s">
         <v>79</v>
       </c>
@@ -1492,7 +1531,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="18" spans="5:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="5:9" x14ac:dyDescent="0.3">
       <c r="H18" t="s">
         <v>81</v>
       </c>
@@ -1500,7 +1539,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="19" spans="5:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="5:9" x14ac:dyDescent="0.3">
       <c r="H19" s="11" t="s">
         <v>82</v>
       </c>
@@ -1508,7 +1547,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="20" spans="5:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="5:9" x14ac:dyDescent="0.3">
       <c r="H20" s="11" t="s">
         <v>83</v>
       </c>
@@ -1516,7 +1555,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="21" spans="5:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="5:9" x14ac:dyDescent="0.3">
       <c r="H21" s="11" t="s">
         <v>84</v>
       </c>
@@ -1524,17 +1563,17 @@
         <v>92</v>
       </c>
     </row>
-    <row r="23" spans="5:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="5:9" x14ac:dyDescent="0.3">
       <c r="I23" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="24" spans="5:9" x14ac:dyDescent="0.35">
+    <row r="24" spans="5:9" x14ac:dyDescent="0.3">
       <c r="I24" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="26" spans="5:9" x14ac:dyDescent="0.35">
+    <row r="26" spans="5:9" x14ac:dyDescent="0.3">
       <c r="I26" t="s">
         <v>95</v>
       </c>
@@ -1547,52 +1586,52 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19B8C298-1B1E-4BB2-871B-BB0A034CE40B}">
   <dimension ref="B2:B14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="123.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="123.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B2" s="14" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B3" s="15" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B4" s="15" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B5" s="14" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B6" s="12" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B7" s="16" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>109</v>
       </c>

</xml_diff>